<commit_message>
docs: atualiza acompanhamento de features whatsapp
</commit_message>
<xml_diff>
--- a/docs/[Lumiz] Calendario Features v1.xlsx
+++ b/docs/[Lumiz] Calendario Features v1.xlsx
@@ -3,11 +3,12 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Features V1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Legenda" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumo Codex 10-06" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Features V1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Legenda" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Features V1'!$B$2:$O$1000</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Features V1'!$B$2:$O$1000</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -16,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -69,8 +70,16 @@
       <b val="1"/>
       <color rgb="004F46E5"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="25">
+  <fills count="31">
     <fill>
       <patternFill/>
     </fill>
@@ -211,8 +220,38 @@
         <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFEB9C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EADCF8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="7">
+  <borders count="8">
     <border/>
     <border>
       <left/>
@@ -265,11 +304,25 @@
         <color rgb="00E5E7EB"/>
       </bottom>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9E2F3"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9E2F3"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9E2F3"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9E2F3"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="79">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -455,6 +508,54 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="24" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="26" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="28" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="29" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="30" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="27" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="26" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="27" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="29" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -732,6 +833,347 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E26"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" style="56" min="1" max="1"/>
+    <col width="24" customWidth="1" style="56" min="2" max="2"/>
+    <col width="70" customWidth="1" style="56" min="3" max="3"/>
+    <col width="34" customWidth="1" style="56" min="4" max="4"/>
+    <col width="22" customWidth="1" style="56" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="56">
+      <c r="A1" s="63" t="inlineStr">
+        <is>
+          <t>Resumo de cobertura WhatsApp-first — Codex 10/06/2026</t>
+        </is>
+      </c>
+      <c r="B1" s="64" t="n"/>
+      <c r="C1" s="64" t="n"/>
+      <c r="D1" s="64" t="n"/>
+      <c r="E1" s="64" t="n"/>
+    </row>
+    <row r="2" ht="24" customHeight="1" s="56">
+      <c r="A2" s="65" t="inlineStr">
+        <is>
+          <t>Escopo atualizado</t>
+        </is>
+      </c>
+      <c r="B2" s="64" t="n"/>
+      <c r="C2" s="64" t="n"/>
+      <c r="D2" s="64" t="n"/>
+      <c r="E2" s="64" t="n"/>
+    </row>
+    <row r="3" ht="24" customHeight="1" s="56">
+      <c r="A3" s="64" t="inlineStr">
+        <is>
+          <t>Inclui comandos Meta/WhatsApp, documentos PDF/foto, contas a pagar, parcelas a receber, gap de caixa, briefing, inventário real estrutural e observabilidade de latência.</t>
+        </is>
+      </c>
+      <c r="B3" s="64" t="n"/>
+      <c r="C3" s="64" t="n"/>
+      <c r="D3" s="64" t="n"/>
+      <c r="E3" s="64" t="n"/>
+    </row>
+    <row r="4" ht="24" customHeight="1" s="56">
+      <c r="A4" s="64" t="n"/>
+      <c r="B4" s="64" t="n"/>
+      <c r="C4" s="64" t="n"/>
+      <c r="D4" s="64" t="n"/>
+      <c r="E4" s="64" t="n"/>
+    </row>
+    <row r="5" ht="24" customHeight="1" s="56">
+      <c r="A5" s="66" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="B5" s="66" t="inlineStr">
+        <is>
+          <t>Quantidade nos itens priorizados</t>
+        </is>
+      </c>
+      <c r="C5" s="66" t="inlineStr">
+        <is>
+          <t>Leitura prática</t>
+        </is>
+      </c>
+      <c r="D5" s="66" t="n"/>
+      <c r="E5" s="66" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1" s="56">
+      <c r="A6" s="67" t="inlineStr">
+        <is>
+          <t>Coberto</t>
+        </is>
+      </c>
+      <c r="B6" s="64" t="n">
+        <v>6</v>
+      </c>
+      <c r="C6" s="64" t="inlineStr">
+        <is>
+          <t>Pronto para teste funcional no WhatsApp.</t>
+        </is>
+      </c>
+      <c r="D6" s="64" t="n"/>
+      <c r="E6" s="64" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1" s="56">
+      <c r="A7" s="68" t="inlineStr">
+        <is>
+          <t>Parcial avançado</t>
+        </is>
+      </c>
+      <c r="B7" s="64" t="n">
+        <v>4</v>
+      </c>
+      <c r="C7" s="64" t="inlineStr">
+        <is>
+          <t>Fluxo principal existe, mas falta etapa complementar ou integração profunda.</t>
+        </is>
+      </c>
+      <c r="D7" s="64" t="n"/>
+      <c r="E7" s="64" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1" s="56">
+      <c r="A8" s="69" t="inlineStr">
+        <is>
+          <t>Parcial</t>
+        </is>
+      </c>
+      <c r="B8" s="64" t="n">
+        <v>10</v>
+      </c>
+      <c r="C8" s="64" t="inlineStr">
+        <is>
+          <t>Base existe, mas depende de configuração, opt-in, dados ou fase posterior.</t>
+        </is>
+      </c>
+      <c r="D8" s="64" t="n"/>
+      <c r="E8" s="64" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1" s="56">
+      <c r="A9" s="70" t="inlineStr">
+        <is>
+          <t>Adiado por decisão de produto</t>
+        </is>
+      </c>
+      <c r="B9" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="64" t="inlineStr">
+        <is>
+          <t>Não implementar agora por decisão operacional/produto.</t>
+        </is>
+      </c>
+      <c r="D9" s="64" t="n"/>
+      <c r="E9" s="64" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1" s="56">
+      <c r="A10" s="71" t="inlineStr">
+        <is>
+          <t>Pendente</t>
+        </is>
+      </c>
+      <c r="B10" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="C10" s="64" t="inlineStr">
+        <is>
+          <t>Ainda não entregue nesta rodada.</t>
+        </is>
+      </c>
+      <c r="D10" s="64" t="n"/>
+      <c r="E10" s="64" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1" s="56">
+      <c r="A11" s="64" t="n"/>
+      <c r="B11" s="64" t="n"/>
+      <c r="C11" s="64" t="n"/>
+      <c r="D11" s="64" t="n"/>
+      <c r="E11" s="64" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1" s="56">
+      <c r="A12" s="64" t="n"/>
+      <c r="B12" s="64" t="n"/>
+      <c r="C12" s="64" t="n"/>
+      <c r="D12" s="64" t="n"/>
+      <c r="E12" s="64" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1" s="56">
+      <c r="A13" s="65" t="inlineStr">
+        <is>
+          <t>Principais testes sugeridos</t>
+        </is>
+      </c>
+      <c r="B13" s="64" t="n"/>
+      <c r="C13" s="64" t="n"/>
+      <c r="D13" s="65" t="inlineStr">
+        <is>
+          <t>Notas de decisão</t>
+        </is>
+      </c>
+      <c r="E13" s="64" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1" s="56">
+      <c r="A14" s="64" t="inlineStr">
+        <is>
+          <t>/ajuda</t>
+        </is>
+      </c>
+      <c r="B14" s="64" t="n"/>
+      <c r="C14" s="64" t="n"/>
+      <c r="D14" s="64" t="inlineStr">
+        <is>
+          <t>Baixa automática de estoque por procedimento não será ativada agora.</t>
+        </is>
+      </c>
+      <c r="E14" s="64" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1" s="56">
+      <c r="A15" s="64" t="inlineStr">
+        <is>
+          <t>/saldo</t>
+        </is>
+      </c>
+      <c r="B15" s="64" t="n"/>
+      <c r="C15" s="64" t="n"/>
+      <c r="D15" s="64" t="inlineStr">
+        <is>
+          <t>A fase futura deve perguntar após procedimento se deseja atualizar estoque.</t>
+        </is>
+      </c>
+      <c r="E15" s="64" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1" s="56">
+      <c r="A16" s="64" t="inlineStr">
+        <is>
+          <t>relatório mês 6</t>
+        </is>
+      </c>
+      <c r="B16" s="64" t="n"/>
+      <c r="C16" s="64" t="n"/>
+      <c r="D16" s="64" t="inlineStr">
+        <is>
+          <t>Quando usuário confirmar, poderá escolher insumos por botão ou texto.</t>
+        </is>
+      </c>
+      <c r="E16" s="64" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1" s="56">
+      <c r="A17" s="64" t="inlineStr">
+        <is>
+          <t>/contas</t>
+        </is>
+      </c>
+      <c r="B17" s="64" t="n"/>
+      <c r="C17" s="64" t="n"/>
+      <c r="D17" s="64" t="inlineStr">
+        <is>
+          <t>WHATSAPP_ASYNC_MEDIA_PROCESSING pode reduzir sensação de demora em PDF/imagem.</t>
+        </is>
+      </c>
+      <c r="E17" s="64" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1" s="56">
+      <c r="A18" s="64" t="inlineStr">
+        <is>
+          <t>/receber</t>
+        </is>
+      </c>
+      <c r="B18" s="64" t="n"/>
+      <c r="C18" s="64" t="n"/>
+      <c r="D18" s="64" t="n"/>
+      <c r="E18" s="64" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1" s="56">
+      <c r="A19" s="64" t="inlineStr">
+        <is>
+          <t>/estoque</t>
+        </is>
+      </c>
+      <c r="B19" s="64" t="n"/>
+      <c r="C19" s="64" t="n"/>
+      <c r="D19" s="64" t="n"/>
+      <c r="E19" s="64" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1" s="56">
+      <c r="A20" s="64" t="inlineStr">
+        <is>
+          <t>configurar estoque</t>
+        </is>
+      </c>
+      <c r="B20" s="64" t="n"/>
+      <c r="C20" s="64" t="n"/>
+      <c r="D20" s="64" t="n"/>
+      <c r="E20" s="64" t="n"/>
+    </row>
+    <row r="21" ht="24" customHeight="1" s="56">
+      <c r="A21" s="64" t="inlineStr">
+        <is>
+          <t>saldo botox</t>
+        </is>
+      </c>
+      <c r="B21" s="64" t="n"/>
+      <c r="C21" s="64" t="n"/>
+      <c r="D21" s="64" t="n"/>
+      <c r="E21" s="64" t="n"/>
+    </row>
+    <row r="22" ht="24" customHeight="1" s="56">
+      <c r="A22" s="64" t="inlineStr">
+        <is>
+          <t>gap de caixa</t>
+        </is>
+      </c>
+      <c r="B22" s="64" t="n"/>
+      <c r="C22" s="64" t="n"/>
+      <c r="D22" s="64" t="n"/>
+      <c r="E22" s="64" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1" s="56">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>briefing</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="24" customHeight="1" s="56">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>validades</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Enviar boleto PDF/foto e confirmar</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Enviar NF de compra e revisar itens detectados</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
@@ -747,8 +1189,8 @@
     <col width="36" customWidth="1" style="56" min="10" max="10"/>
     <col width="52" customWidth="1" style="56" min="11" max="11"/>
     <col width="102.86" customWidth="1" style="56" min="12" max="12"/>
-    <col width="18" customWidth="1" style="56" min="13" max="26"/>
-    <col width="58" customWidth="1" style="56" min="14" max="14"/>
+    <col width="22" customWidth="1" style="56" min="13" max="26"/>
+    <col width="72" customWidth="1" style="56" min="14" max="14"/>
     <col width="42" customWidth="1" style="56" min="15" max="15"/>
   </cols>
   <sheetData>
@@ -767,7 +1209,7 @@
       <c r="L1" s="1" t="n"/>
       <c r="M1" s="57" t="inlineStr">
         <is>
-          <t>Atualizado por Codex em 03/06/2026: cobertura WhatsApp-first</t>
+          <t>Atualizado por Codex em 10/06/2026: WhatsApp-first + inventario real + observabilidade</t>
         </is>
       </c>
       <c r="N1" s="1" t="n"/>
@@ -841,17 +1283,17 @@
           <t>Status e prazo</t>
         </is>
       </c>
-      <c r="M2" s="58" t="inlineStr">
-        <is>
-          <t>Status Codex 03/06</t>
-        </is>
-      </c>
-      <c r="N2" s="58" t="inlineStr">
+      <c r="M2" s="72" t="inlineStr">
+        <is>
+          <t>Status Codex 10/06</t>
+        </is>
+      </c>
+      <c r="N2" s="72" t="inlineStr">
         <is>
           <t>Cobertura WhatsApp atual</t>
         </is>
       </c>
-      <c r="O2" s="58" t="inlineStr">
+      <c r="O2" s="72" t="inlineStr">
         <is>
           <t>Teste WhatsApp sugerido</t>
         </is>
@@ -923,19 +1365,19 @@
           <t>ok</t>
         </is>
       </c>
-      <c r="M3" s="59" t="inlineStr">
+      <c r="M3" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N3" s="60" t="inlineStr">
         <is>
-          <t>Receita por texto com extracao, resumo e confirmacao antes de registrar.</t>
+          <t>Receita por texto com extração, resumo e confirmação antes de registrar. Pós-onboarding não pede mais ativação de modo real.</t>
         </is>
       </c>
       <c r="O3" s="60" t="inlineStr">
         <is>
-          <t>Romulo botox hoje 12000 em 6x</t>
+          <t>Romulo botox hoje 12000 em 6x -&gt; 1</t>
         </is>
       </c>
       <c r="P3" s="1" t="n"/>
@@ -1005,19 +1447,19 @@
           <t>configurando / pausado. 2 dias</t>
         </is>
       </c>
-      <c r="M4" s="61" t="inlineStr">
+      <c r="M4" s="74" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
       <c r="N4" s="60" t="inlineStr">
         <is>
-          <t>Audio nao foi coberto nesta rodada WhatsApp-first.</t>
+          <t>Áudio não foi tratado como entrega fechada desta rodada. Há pontos de observabilidade para transcrição, mas precisa teste/validação dedicada.</t>
         </is>
       </c>
       <c r="O4" s="60" t="inlineStr">
         <is>
-          <t>Enviar audio com venda/despesa quando STT estiver ativo</t>
+          <t>Enviar áudio curto com venda quando a fase de áudio for retomada</t>
         </is>
       </c>
       <c r="P4" s="1" t="n"/>
@@ -1087,19 +1529,19 @@
           <t xml:space="preserve">ending points - finalizando. 03/06 ver se ta rolando </t>
         </is>
       </c>
-      <c r="M5" s="62" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="M5" s="75" t="inlineStr">
+        <is>
+          <t>Parcial avançado</t>
         </is>
       </c>
       <c r="N5" s="60" t="inlineStr">
         <is>
-          <t>Forma de pagamento e parcelamento por texto cobertos; parcelas alimentam recebiveis.</t>
+          <t>Forma de pagamento e parcelamento por texto cobertos; vendas parceladas alimentam parcelas a receber. Rastreio fino por credenciadora ainda depende de MDR/Alter.</t>
         </is>
       </c>
       <c r="O5" s="60" t="inlineStr">
         <is>
-          <t>Romulo botox hoje 12000 em 6x</t>
+          <t>Botox 12000 crédito em 6x -&gt; /receber</t>
         </is>
       </c>
       <c r="P5" s="1" t="n"/>
@@ -1169,19 +1611,19 @@
           <t>só bandeira pela alter. taxa da maquininha o usuario coloca (add isso no onboarding)</t>
         </is>
       </c>
-      <c r="M6" s="62" t="inlineStr">
+      <c r="M6" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N6" s="60" t="inlineStr">
         <is>
-          <t>Recebiveis por parcelas cobertos; rastreio profundo por credenciadora/Alter ainda pendente.</t>
+          <t>Recebíveis por parcelas cobertos no WhatsApp. Credenciadora, taxa, data líquida real e status Alter ainda ficam para integração financeira posterior.</t>
         </is>
       </c>
       <c r="O6" s="60" t="inlineStr">
         <is>
-          <t>parcelas a receber</t>
+          <t>/receber</t>
         </is>
       </c>
       <c r="P6" s="1" t="n"/>
@@ -1251,19 +1693,19 @@
           <t xml:space="preserve">configurando - finalizando. 03/06 ver se ta rolando </t>
         </is>
       </c>
-      <c r="M7" s="59" t="inlineStr">
+      <c r="M7" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N7" s="60" t="inlineStr">
         <is>
-          <t>Consulta rapida via saldo, relatorio e stats/receita quando houver dados.</t>
+          <t>Consulta rápida via /saldo, /relatorio, relatório por mês e briefing manual, usando dados reais registrados.</t>
         </is>
       </c>
       <c r="O7" s="60" t="inlineStr">
         <is>
-          <t>/saldo</t>
+          <t>/saldo ou relatório mês 6</t>
         </is>
       </c>
       <c r="P7" s="1" t="n"/>
@@ -1333,19 +1775,19 @@
           <t>Pronto ✅</t>
         </is>
       </c>
-      <c r="M8" s="59" t="inlineStr">
+      <c r="M8" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N8" s="60" t="inlineStr">
         <is>
-          <t>Boleto por PDF/foto entra no fluxo de documento com confirmacao.</t>
+          <t>PDF/foto de boleto entra no fluxo de documento, mostra resumo limpo, exige confirmação/correção/cancelamento e registra conta a pagar com rastreabilidade.</t>
         </is>
       </c>
       <c r="O8" s="60" t="inlineStr">
         <is>
-          <t>Enviar boleto em PDF e responder 1</t>
+          <t>Enviar boleto PDF/foto -&gt; Confirmar</t>
         </is>
       </c>
       <c r="P8" s="1" t="n"/>
@@ -1415,19 +1857,19 @@
           <t>Pronto ✅ - Ajustar leitura para pegar a quantidade e valor de cada produto (caso NF tenha mais de um produto)</t>
         </is>
       </c>
-      <c r="M9" s="62" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="M9" s="75" t="inlineStr">
+        <is>
+          <t>Parcial avançado</t>
         </is>
       </c>
       <c r="N9" s="60" t="inlineStr">
         <is>
-          <t>NF/documento coberto para leitura principal; itemizacao detalhada por produto ainda pendente.</t>
+          <t>NF/documento por PDF/foto lê fornecedor, total, vencimento e tenta itemização. Itens só alimentam inventário real quando casam com produto já cadastrado, evitando catálogo sujo.</t>
         </is>
       </c>
       <c r="O9" s="60" t="inlineStr">
         <is>
-          <t>Enviar NF em PDF/foto</t>
+          <t>Enviar NF de compra com itens -&gt; revisar confirmação</t>
         </is>
       </c>
       <c r="P9" s="1" t="n"/>
@@ -1566,14 +2008,14 @@
 por audio stand by por agora</t>
         </is>
       </c>
-      <c r="M11" s="62" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="M11" s="75" t="inlineStr">
+        <is>
+          <t>Parcial avançado</t>
         </is>
       </c>
       <c r="N11" s="60" t="inlineStr">
         <is>
-          <t>Despesa por texto coberta, incluindo recorrencia explicita; audio segue pendente.</t>
+          <t>Despesa por texto coberta, inclusive conta a pagar e recorrência explícita. Áudio ainda não entra como entrega final.</t>
         </is>
       </c>
       <c r="O11" s="60" t="inlineStr">
@@ -1644,19 +2086,19 @@
         </is>
       </c>
       <c r="L12" s="27" t="n"/>
-      <c r="M12" s="62" t="inlineStr">
+      <c r="M12" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N12" s="60" t="inlineStr">
         <is>
-          <t>Categorizacao automatica via heuristica/IA em textos e documentos; refinamento continuo.</t>
+          <t>Categorização automática por heurística/IA em textos e documentos; correções manuais já são aceitas, mas aprendizado persistente ainda não é fase fechada.</t>
         </is>
       </c>
       <c r="O12" s="60" t="inlineStr">
         <is>
-          <t>toxina 600 no pix</t>
+          <t>toxina 600 no pix -&gt; corrigir categoria se necessário</t>
         </is>
       </c>
       <c r="P12" s="1" t="n"/>
@@ -1722,19 +2164,19 @@
           <t>configurando. 03/06</t>
         </is>
       </c>
-      <c r="M13" s="62" t="inlineStr">
+      <c r="M13" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N13" s="60" t="inlineStr">
         <is>
-          <t>Contas proximas aparecem em contas a pagar/briefing; alerta automatico depende de env e opt-in.</t>
+          <t>Contas próximas aparecem em /contas e briefing. Alertas automáticos dependem de env/cron e opt-in por perfil.</t>
         </is>
       </c>
       <c r="O13" s="60" t="inlineStr">
         <is>
-          <t>/contas</t>
+          <t>/contas ou briefing</t>
         </is>
       </c>
       <c r="P13" s="1" t="n"/>
@@ -2398,19 +2840,19 @@
           <t>Ja le o valor e o nome do produto - Ajustar leitura para pegar a quantidade e valor de cada produto (caso NF tenha mais de um produto). Uma semana. Começando dia 08/06</t>
         </is>
       </c>
-      <c r="M23" s="62" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="M23" s="75" t="inlineStr">
+        <is>
+          <t>Parcial avançado</t>
         </is>
       </c>
       <c r="N23" s="60" t="inlineStr">
         <is>
-          <t>Entrada via documento existe, mas quantidade/valor por item ainda precisa refinamento.</t>
+          <t>Entrada via NF/documento está integrada ao inventário real somente para produtos existentes. Cadastro inicial do estoque pode ser feito por lista no WhatsApp.</t>
         </is>
       </c>
       <c r="O23" s="60" t="inlineStr">
         <is>
-          <t>Enviar NF de compra</t>
+          <t>configurar estoque; depois enviar NF de compra</t>
         </is>
       </c>
       <c r="P23" s="1" t="n"/>
@@ -2546,19 +2988,19 @@
           <t>Fazer. Colocar lista manual do estoque atual via wpp. Um vez feito, ja começa a rodar.  Começando dia 08/06</t>
         </is>
       </c>
-      <c r="M25" s="62" t="inlineStr">
-        <is>
-          <t>Parcial</t>
+      <c r="M25" s="77" t="inlineStr">
+        <is>
+          <t>Adiado por decisão de produto</t>
         </is>
       </c>
       <c r="N25" s="60" t="inlineStr">
         <is>
-          <t>Baixa manual por WhatsApp coberta; baixa automatica por procedimento ainda pendente.</t>
+          <t>Não haverá baixa automática por procedimento agora. Estrutura técnica existe, mas o fluxo público será confirmação pós-procedimento antes de atualizar estoque.</t>
         </is>
       </c>
       <c r="O25" s="60" t="inlineStr">
         <is>
-          <t>baixar estoque botox 2 unidades</t>
+          <t>Sem teste público nesta fase</t>
         </is>
       </c>
       <c r="P25" s="1" t="n"/>
@@ -2694,14 +3136,14 @@
           <t>Opção de add validade do produto quando registrar entrada de estoque</t>
         </is>
       </c>
-      <c r="M27" s="62" t="inlineStr">
+      <c r="M27" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N27" s="60" t="inlineStr">
         <is>
-          <t>Consulta validades e endpoint de alerta operacional cobertos; depende de dados de validade.</t>
+          <t>Validades podem ser consultadas e usadas em alerta quando houver validade cadastrada ou extraída de documentos.</t>
         </is>
       </c>
       <c r="O27" s="60" t="inlineStr">
@@ -2776,14 +3218,14 @@
           <t>Stand By</t>
         </is>
       </c>
-      <c r="M28" s="62" t="inlineStr">
+      <c r="M28" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N28" s="60" t="inlineStr">
         <is>
-          <t>Alertas de estoque baixo existem; minimo adaptativo ainda nao concluido.</t>
+          <t>Estoque baixo aparece em /estoque e briefing; mínimo adaptativo automático ainda não está concluído.</t>
         </is>
       </c>
       <c r="O28" s="60" t="inlineStr">
@@ -2924,19 +3366,19 @@
           <t>Stand By</t>
         </is>
       </c>
-      <c r="M30" s="61" t="inlineStr">
-        <is>
-          <t>Pendente</t>
+      <c r="M30" s="78" t="inlineStr">
+        <is>
+          <t>Parcial</t>
         </is>
       </c>
       <c r="N30" s="60" t="inlineStr">
         <is>
-          <t>Inventario periodico assistido nao foi implementado nesta rodada.</t>
+          <t>Inventário real estrutural criado: cadastro inicial por lista no WhatsApp, produtos, lotes e movimentos. Inventário periódico/recontagem assistida ainda fica para próxima fase.</t>
         </is>
       </c>
       <c r="O30" s="60" t="inlineStr">
         <is>
-          <t>Pendente</t>
+          <t>configurar estoque</t>
         </is>
       </c>
       <c r="P30" s="1" t="n"/>
@@ -3006,14 +3448,14 @@
           <t>Stand By</t>
         </is>
       </c>
-      <c r="M31" s="59" t="inlineStr">
+      <c r="M31" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N31" s="60" t="inlineStr">
         <is>
-          <t>Consulta de saldo por produto via WhatsApp coberta.</t>
+          <t>Consulta de estoque geral e saldo por produto usa inventário real primeiro e cai para modelo legado quando necessário.</t>
         </is>
       </c>
       <c r="O31" s="60" t="inlineStr">
@@ -4222,14 +4664,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M49" s="59" t="inlineStr">
+      <c r="M49" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N49" s="60" t="inlineStr">
         <is>
-          <t>Saldo disponivel ajustado para base de caixa e consultavel por WhatsApp.</t>
+          <t>Saldo disponível em tempo real ajustado para base de caixa e consultável por WhatsApp.</t>
         </is>
       </c>
       <c r="O49" s="60" t="inlineStr">
@@ -4370,14 +4812,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M51" s="59" t="inlineStr">
+      <c r="M51" s="73" t="inlineStr">
         <is>
           <t>Coberto</t>
         </is>
       </c>
       <c r="N51" s="60" t="inlineStr">
         <is>
-          <t>Gap de caixa dos proximos 30 dias disponivel por comando.</t>
+          <t>Gap de caixa dos próximos 30 dias disponível por comando, considerando entradas/saídas previstas disponíveis.</t>
         </is>
       </c>
       <c r="O51" s="60" t="inlineStr">
@@ -4716,14 +5158,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M56" s="62" t="inlineStr">
+      <c r="M56" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N56" s="60" t="inlineStr">
         <is>
-          <t>Briefing manual e endpoint opt-in cobertos; disparo automatico depende de env/cron.</t>
+          <t>Briefing manual e endpoint operacional existem. Envio automático depende de ativar envs, cron e opt-in do perfil.</t>
         </is>
       </c>
       <c r="O56" s="60" t="inlineStr">
@@ -4798,14 +5240,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M57" s="62" t="inlineStr">
+      <c r="M57" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N57" s="60" t="inlineStr">
         <is>
-          <t>Gap de caixa coberto; sugestao Alter ainda pendente.</t>
+          <t>Gap de caixa coberto; sugestão Alter específica ainda depende da integração Alter real.</t>
         </is>
       </c>
       <c r="O57" s="60" t="inlineStr">
@@ -4880,14 +5322,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M58" s="62" t="inlineStr">
+      <c r="M58" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N58" s="60" t="inlineStr">
         <is>
-          <t>Estoque critico aparece em estoque/briefing; proatividade depende de opt-in/cron.</t>
+          <t>Estoque crítico aparece em /estoque e briefing. Proatividade automática depende de cron/opt-in.</t>
         </is>
       </c>
       <c r="O58" s="60" t="inlineStr">
@@ -4962,14 +5404,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M59" s="62" t="inlineStr">
+      <c r="M59" s="76" t="inlineStr">
         <is>
           <t>Parcial</t>
         </is>
       </c>
       <c r="N59" s="60" t="inlineStr">
         <is>
-          <t>Validades por consulta e endpoint opt-in cobertas.</t>
+          <t>Consulta e endpoint de alertas de validade existem; automação depende de dados de validade e opt-in.</t>
         </is>
       </c>
       <c r="O59" s="60" t="inlineStr">
@@ -5176,14 +5618,14 @@
           <t>Realizar</t>
         </is>
       </c>
-      <c r="M62" s="61" t="inlineStr">
+      <c r="M62" s="74" t="inlineStr">
         <is>
           <t>Pendente</t>
         </is>
       </c>
       <c r="N62" s="60" t="inlineStr">
         <is>
-          <t>Alerta de inadimplencia nao foi implementado nesta rodada.</t>
+          <t>Alerta de inadimplência não foi implementado nesta rodada WhatsApp-first.</t>
         </is>
       </c>
       <c r="O62" s="60" t="inlineStr">
@@ -32408,7 +32850,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>